<commit_message>
feat: Synchronize all 30 Rakhi Startup Bazaar stalls with Supabase schema & seeder
</commit_message>
<xml_diff>
--- a/client/src/rakhi-stalls.xlsx
+++ b/client/src/rakhi-stalls.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="312">
   <si>
     <t>Timestamp</t>
   </si>
@@ -750,6 +750,174 @@
   </si>
   <si>
     <t>https://drive.google.com/open?id=1dzckh-h1yPfKdVnFkzaCsK_m9rhVfJRN</t>
+  </si>
+  <si>
+    <t>Saptarshi Kundu</t>
+  </si>
+  <si>
+    <t>saptarshi1.kundu@stu.adamasuniversity.ac.in</t>
+  </si>
+  <si>
+    <t>Charmnco</t>
+  </si>
+  <si>
+    <t>Our stall offers a curated collection of cute, trendy, and affordable accessories, including jewellery, bracelets, hair clutches/claw clips, and other stylish little essentials. Perfect for adding a simple touch of charm to your everyday look or gifting someone special.</t>
+  </si>
+  <si>
+    <t>@charmnco.official</t>
+  </si>
+  <si>
+    <t>T2608251408397415476310</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1Ol5_dLg9PiIrs7AaUO3Tw9cVKKDMgwN7</t>
+  </si>
+  <si>
+    <t>Prapti Biswas</t>
+  </si>
+  <si>
+    <t>prapti.biswas@stu.adamasuniversity.ac.in</t>
+  </si>
+  <si>
+    <t>BSc Forensic Science</t>
+  </si>
+  <si>
+    <t>Faces and Fun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Face Painting </t>
+  </si>
+  <si>
+    <t>maybe, min 2</t>
+  </si>
+  <si>
+    <t>under a fan for fast drying, near a water source</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1Pj-_MyLlY3km7IKi7XftbZuvViqio8Tp</t>
+  </si>
+  <si>
+    <t>Disha Saha</t>
+  </si>
+  <si>
+    <t>disha2.saha@stu.adamasuniversity.ac.in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chemistry </t>
+  </si>
+  <si>
+    <t>Sobas</t>
+  </si>
+  <si>
+    <t>Bloom with Clay</t>
+  </si>
+  <si>
+    <t>We will sell sustainable decorated pots with plants and sustainable candles</t>
+  </si>
+  <si>
+    <t>Null</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1io6yHjgTNXds42JPVpeB7L2CTXDg1HI9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saptarnab Karmakar </t>
+  </si>
+  <si>
+    <t>saptarnab1.karmakar@stu.adamasuniversity.ac.in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Environmental science and sustainability </t>
+  </si>
+  <si>
+    <t>আবার খাবো</t>
+  </si>
+  <si>
+    <t>Homemade food</t>
+  </si>
+  <si>
+    <t>6289091985-2@ybl</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1-mbtnVYAxb54_Xe1RdUnOU_EFxIWAoyx</t>
+  </si>
+  <si>
+    <t>Debjeet Kundu</t>
+  </si>
+  <si>
+    <t>debjeet1.kundu@stu.adamasuniversity.ac.in</t>
+  </si>
+  <si>
+    <t>Kissewala: Film and Drama Club</t>
+  </si>
+  <si>
+    <t>Creative reels and story making</t>
+  </si>
+  <si>
+    <t>kissewalaofcl_au</t>
+  </si>
+  <si>
+    <t>Nah</t>
+  </si>
+  <si>
+    <t>One shelf</t>
+  </si>
+  <si>
+    <t>NEFe7d8982f8af742319f79722037efd670</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1V9Ll7fy9FRPixOJpJ7m33BePNzSNwmHr</t>
+  </si>
+  <si>
+    <t>Ishita Das</t>
+  </si>
+  <si>
+    <t>ishita2.das@stu.adamasuniversity.ac.in</t>
+  </si>
+  <si>
+    <t>Chemistry</t>
+  </si>
+  <si>
+    <t>School of Basic and Applied Sciences</t>
+  </si>
+  <si>
+    <t>Swaad and Sehat</t>
+  </si>
+  <si>
+    <t>We will be selling homemade healthy snacks along with handmade, creative bookmarks</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1nb3YQhUpdsqOlBqsvjx7MZPmSMwoJHuF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RINI KARAK </t>
+  </si>
+  <si>
+    <t>rini2.karak@stu.adamasuniversity.ac.in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GEOGRAPHY </t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOBAS </t>
+  </si>
+  <si>
+    <t>Momolicious!</t>
+  </si>
+  <si>
+    <t>Momo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extension cords </t>
+  </si>
+  <si>
+    <t>6290406354@ybl</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=154FlnefKWhHur3_9jJwbM5kNL3BMkXyt</t>
   </si>
   <si>
     <t xml:space="preserve">Aaditya Singh </t>
@@ -960,7 +1128,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:S24" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:S31" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="19">
     <tableColumn name="Timestamp" id="1"/>
     <tableColumn name="Full Name" id="2"/>
@@ -1200,7 +1368,8 @@
     <col customWidth="1" min="16" max="16" width="21.13"/>
     <col customWidth="1" min="17" max="17" width="22.25"/>
     <col customWidth="1" min="18" max="18" width="25.88"/>
-    <col customWidth="1" min="19" max="25" width="18.88"/>
+    <col customWidth="1" min="19" max="19" width="56.25"/>
+    <col customWidth="1" min="20" max="25" width="18.88"/>
   </cols>
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
@@ -2230,63 +2399,69 @@
       </c>
     </row>
     <row r="18" ht="22.5" customHeight="1">
-      <c r="A18" s="11">
+      <c r="A18" s="6">
         <v>46259.466084942134</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="C18" s="12" t="s">
+      <c r="C18" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="D18" s="12">
+      <c r="D18" s="7">
         <v>9.073399316E9</v>
       </c>
-      <c r="E18" s="12" t="s">
+      <c r="E18" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="F18" s="12" t="s">
+      <c r="F18" s="7" t="s">
         <v>190</v>
       </c>
-      <c r="G18" s="12" t="s">
+      <c r="G18" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="H18" s="12" t="s">
+      <c r="H18" s="7" t="s">
         <v>191</v>
       </c>
-      <c r="I18" s="12">
+      <c r="I18" s="7">
         <v>2.0</v>
       </c>
-      <c r="J18" s="12" t="s">
+      <c r="J18" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="K18" s="12" t="s">
+      <c r="K18" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="L18" s="12" t="s">
+      <c r="L18" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="M18" s="12" t="s">
+      <c r="M18" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="N18" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="O18" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="P18" s="12" t="s">
+      <c r="N18" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="O18" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="P18" s="7" t="s">
         <v>194</v>
       </c>
-      <c r="Q18" s="12">
+      <c r="Q18" s="7">
         <v>3.1319535913E11</v>
       </c>
-      <c r="R18" s="13" t="s">
+      <c r="R18" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="S18" s="12" t="s">
+      <c r="S18" s="7" t="s">
         <v>34</v>
       </c>
+      <c r="T18" s="9"/>
+      <c r="U18" s="9"/>
+      <c r="V18" s="9"/>
+      <c r="W18" s="9"/>
+      <c r="X18" s="9"/>
+      <c r="Y18" s="9"/>
     </row>
     <row r="19" ht="22.5" customHeight="1">
       <c r="A19" s="11">
@@ -2348,295 +2523,714 @@
       </c>
     </row>
     <row r="20" ht="22.5" customHeight="1">
-      <c r="A20" s="11">
+      <c r="A20" s="6">
         <v>46259.5162468287</v>
       </c>
-      <c r="B20" s="12" t="s">
+      <c r="B20" s="7" t="s">
         <v>206</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="C20" s="7" t="s">
         <v>207</v>
       </c>
-      <c r="D20" s="12">
+      <c r="D20" s="7">
         <v>6.290860133E9</v>
       </c>
-      <c r="E20" s="12" t="s">
+      <c r="E20" s="7" t="s">
         <v>208</v>
       </c>
-      <c r="F20" s="12" t="s">
+      <c r="F20" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="G20" s="12" t="s">
+      <c r="G20" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="H20" s="12" t="s">
+      <c r="H20" s="7" t="s">
         <v>209</v>
       </c>
-      <c r="I20" s="12">
+      <c r="I20" s="7">
         <v>3.0</v>
       </c>
-      <c r="J20" s="12" t="s">
+      <c r="J20" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="K20" s="12" t="s">
+      <c r="K20" s="7" t="s">
         <v>210</v>
       </c>
-      <c r="L20" s="12" t="s">
+      <c r="L20" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="M20" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="N20" s="12" t="s">
+      <c r="M20" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="N20" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="O20" s="12" t="s">
+      <c r="O20" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="P20" s="12" t="s">
+      <c r="P20" s="7" t="s">
         <v>214</v>
       </c>
-      <c r="Q20" s="12" t="s">
+      <c r="Q20" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="R20" s="13" t="s">
+      <c r="R20" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="S20" s="12" t="s">
+      <c r="S20" s="7" t="s">
         <v>34</v>
       </c>
+      <c r="T20" s="9"/>
+      <c r="U20" s="9"/>
+      <c r="V20" s="9"/>
+      <c r="W20" s="9"/>
+      <c r="X20" s="9"/>
+      <c r="Y20" s="9"/>
     </row>
     <row r="21" ht="22.5" customHeight="1">
-      <c r="A21" s="11">
+      <c r="A21" s="6">
         <v>46259.52240210648</v>
       </c>
-      <c r="B21" s="12" t="s">
+      <c r="B21" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="C21" s="12" t="s">
+      <c r="C21" s="7" t="s">
         <v>218</v>
       </c>
-      <c r="D21" s="12">
+      <c r="D21" s="7">
         <v>8.509482008E9</v>
       </c>
-      <c r="E21" s="12" t="s">
+      <c r="E21" s="7" t="s">
         <v>219</v>
       </c>
-      <c r="F21" s="12" t="s">
+      <c r="F21" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="G21" s="12" t="s">
+      <c r="G21" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="H21" s="12" t="s">
+      <c r="H21" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="I21" s="12">
+      <c r="I21" s="7">
         <v>3.0</v>
       </c>
-      <c r="J21" s="12" t="s">
+      <c r="J21" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="K21" s="12" t="s">
+      <c r="K21" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="L21" s="12" t="s">
+      <c r="L21" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="M21" s="12" t="s">
+      <c r="M21" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="N21" s="12" t="s">
+      <c r="N21" s="7" t="s">
         <v>222</v>
       </c>
-      <c r="O21" s="12" t="s">
+      <c r="O21" s="7" t="s">
         <v>222</v>
       </c>
-      <c r="P21" s="12" t="s">
+      <c r="P21" s="7" t="s">
         <v>223</v>
       </c>
-      <c r="Q21" s="12" t="s">
+      <c r="Q21" s="7" t="s">
         <v>224</v>
       </c>
-      <c r="R21" s="13" t="s">
+      <c r="R21" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="S21" s="12" t="s">
+      <c r="S21" s="7" t="s">
         <v>34</v>
       </c>
+      <c r="T21" s="9"/>
+      <c r="U21" s="9"/>
+      <c r="V21" s="9"/>
+      <c r="W21" s="9"/>
+      <c r="X21" s="9"/>
+      <c r="Y21" s="9"/>
     </row>
     <row r="22" ht="22.5" customHeight="1">
-      <c r="A22" s="11">
+      <c r="A22" s="6">
         <v>46259.523050821765</v>
       </c>
-      <c r="B22" s="12" t="s">
+      <c r="B22" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="C22" s="12" t="s">
+      <c r="C22" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="D22" s="12">
+      <c r="D22" s="7">
         <v>7.478069398E9</v>
       </c>
-      <c r="E22" s="12" t="s">
+      <c r="E22" s="7" t="s">
         <v>228</v>
       </c>
-      <c r="F22" s="12" t="s">
+      <c r="F22" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="G22" s="12" t="s">
+      <c r="G22" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="H22" s="12" t="s">
+      <c r="H22" s="7" t="s">
         <v>229</v>
       </c>
-      <c r="I22" s="12">
+      <c r="I22" s="7">
         <v>3.0</v>
       </c>
-      <c r="J22" s="12" t="s">
+      <c r="J22" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="K22" s="12" t="s">
+      <c r="K22" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="L22" s="12" t="s">
+      <c r="L22" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="M22" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="N22" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="O22" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="P22" s="12" t="s">
+      <c r="M22" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="N22" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="O22" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="P22" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="Q22" s="12" t="s">
+      <c r="Q22" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="R22" s="13" t="s">
+      <c r="R22" s="8" t="s">
         <v>233</v>
       </c>
-      <c r="S22" s="12" t="s">
+      <c r="S22" s="7" t="s">
         <v>34</v>
       </c>
+      <c r="T22" s="9"/>
+      <c r="U22" s="9"/>
+      <c r="V22" s="9"/>
+      <c r="W22" s="9"/>
+      <c r="X22" s="9"/>
+      <c r="Y22" s="9"/>
     </row>
     <row r="23" ht="22.5" customHeight="1">
-      <c r="A23" s="11">
+      <c r="A23" s="6">
         <v>46259.52523162037</v>
       </c>
-      <c r="B23" s="12" t="s">
+      <c r="B23" s="7" t="s">
         <v>234</v>
       </c>
-      <c r="C23" s="12" t="s">
+      <c r="C23" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="D23" s="12">
+      <c r="D23" s="7">
         <v>9.332305435E9</v>
       </c>
-      <c r="E23" s="12" t="s">
+      <c r="E23" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="F23" s="12" t="s">
+      <c r="F23" s="7" t="s">
         <v>237</v>
       </c>
-      <c r="G23" s="12" t="s">
+      <c r="G23" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="H23" s="12" t="s">
+      <c r="H23" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="I23" s="12">
+      <c r="I23" s="7">
         <v>3.0</v>
       </c>
-      <c r="J23" s="12" t="s">
+      <c r="J23" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="K23" s="12" t="s">
+      <c r="K23" s="7" t="s">
         <v>239</v>
       </c>
-      <c r="L23" s="13" t="s">
+      <c r="L23" s="8" t="s">
         <v>240</v>
       </c>
-      <c r="M23" s="12" t="s">
+      <c r="M23" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="N23" s="12" t="s">
+      <c r="N23" s="7" t="s">
         <v>241</v>
       </c>
-      <c r="O23" s="12" t="s">
+      <c r="O23" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="P23" s="12" t="s">
+      <c r="P23" s="7" t="s">
         <v>243</v>
       </c>
-      <c r="Q23" s="12" t="s">
+      <c r="Q23" s="7" t="s">
         <v>244</v>
       </c>
-      <c r="R23" s="13" t="s">
+      <c r="R23" s="8" t="s">
         <v>245</v>
       </c>
-      <c r="S23" s="12" t="s">
+      <c r="S23" s="7" t="s">
         <v>34</v>
       </c>
+      <c r="T23" s="9"/>
+      <c r="U23" s="9"/>
+      <c r="V23" s="9"/>
+      <c r="W23" s="9"/>
+      <c r="X23" s="9"/>
+      <c r="Y23" s="9"/>
     </row>
     <row r="24" ht="22.5" customHeight="1">
-      <c r="A24" s="2">
+      <c r="A24" s="11">
+        <v>46259.698406701384</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>246</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D24" s="12">
+        <v>9.33025086E9</v>
+      </c>
+      <c r="E24" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F24" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="G24" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="H24" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="I24" s="12">
+        <v>2.0</v>
+      </c>
+      <c r="J24" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="K24" s="12" t="s">
+        <v>249</v>
+      </c>
+      <c r="L24" s="12" t="s">
+        <v>250</v>
+      </c>
+      <c r="M24" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="N24" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="O24" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="P24" s="12">
+        <v>299.0</v>
+      </c>
+      <c r="Q24" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="R24" s="13" t="s">
+        <v>252</v>
+      </c>
+      <c r="S24" s="12" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="25" ht="22.5" customHeight="1">
+      <c r="A25" s="11">
+        <v>46259.704018958335</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>254</v>
+      </c>
+      <c r="D25" s="12">
+        <v>9.051625436E9</v>
+      </c>
+      <c r="E25" s="12" t="s">
+        <v>255</v>
+      </c>
+      <c r="F25" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="G25" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="H25" s="12" t="s">
+        <v>256</v>
+      </c>
+      <c r="I25" s="12">
+        <v>2.0</v>
+      </c>
+      <c r="J25" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="K25" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="M25" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="N25" s="12" t="s">
+        <v>258</v>
+      </c>
+      <c r="O25" s="12" t="s">
+        <v>259</v>
+      </c>
+      <c r="P25" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="Q25" s="12">
+        <v>6.60344939556E11</v>
+      </c>
+      <c r="R25" s="13" t="s">
+        <v>261</v>
+      </c>
+      <c r="S25" s="12" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="26" ht="22.5" customHeight="1">
+      <c r="A26" s="11">
+        <v>46259.86789954861</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>263</v>
+      </c>
+      <c r="D26" s="12">
+        <v>7.439299433E9</v>
+      </c>
+      <c r="E26" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="F26" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="H26" s="12" t="s">
+        <v>266</v>
+      </c>
+      <c r="I26" s="12">
+        <v>3.0</v>
+      </c>
+      <c r="J26" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="K26" s="12" t="s">
+        <v>267</v>
+      </c>
+      <c r="L26" s="12" t="s">
+        <v>268</v>
+      </c>
+      <c r="M26" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="N26" s="12">
+        <v>2.0</v>
+      </c>
+      <c r="P26" s="12">
+        <v>299.0</v>
+      </c>
+      <c r="Q26" s="12">
+        <v>6.60394470865E11</v>
+      </c>
+      <c r="R26" s="13" t="s">
+        <v>269</v>
+      </c>
+      <c r="S26" s="12" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="27" ht="22.5" customHeight="1">
+      <c r="A27" s="11">
+        <v>46259.87033831018</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="D27" s="12">
+        <v>6.289091985E9</v>
+      </c>
+      <c r="E27" s="12" t="s">
+        <v>272</v>
+      </c>
+      <c r="F27" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="G27" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="H27" s="12" t="s">
+        <v>273</v>
+      </c>
+      <c r="I27" s="12">
+        <v>3.0</v>
+      </c>
+      <c r="J27" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="K27" s="12" t="s">
+        <v>274</v>
+      </c>
+      <c r="M27" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="N27" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="O27" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="P27" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="Q27" s="12" t="s">
+        <v>275</v>
+      </c>
+      <c r="R27" s="13" t="s">
+        <v>276</v>
+      </c>
+      <c r="S27" s="12" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="28" ht="22.5" customHeight="1">
+      <c r="A28" s="11">
+        <v>46259.881440428246</v>
+      </c>
+      <c r="B28" s="12" t="s">
+        <v>277</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>278</v>
+      </c>
+      <c r="D28" s="12">
+        <v>9.073304565E9</v>
+      </c>
+      <c r="E28" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F28" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="G28" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="H28" s="12" t="s">
+        <v>279</v>
+      </c>
+      <c r="I28" s="12">
+        <v>3.0</v>
+      </c>
+      <c r="J28" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="K28" s="12" t="s">
+        <v>280</v>
+      </c>
+      <c r="L28" s="12" t="s">
+        <v>281</v>
+      </c>
+      <c r="M28" s="12" t="s">
+        <v>282</v>
+      </c>
+      <c r="N28" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="O28" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="P28" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="Q28" s="12" t="s">
+        <v>284</v>
+      </c>
+      <c r="R28" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="S28" s="12" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="29" ht="22.5" customHeight="1">
+      <c r="A29" s="11">
+        <v>46259.93994625</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>286</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>287</v>
+      </c>
+      <c r="D29" s="12">
+        <v>7.04422899E9</v>
+      </c>
+      <c r="E29" s="12" t="s">
+        <v>288</v>
+      </c>
+      <c r="F29" s="12" t="s">
+        <v>289</v>
+      </c>
+      <c r="G29" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="H29" s="12" t="s">
+        <v>290</v>
+      </c>
+      <c r="I29" s="12">
+        <v>3.0</v>
+      </c>
+      <c r="J29" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="K29" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="M29" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="N29" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="P29" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="Q29" s="12">
+        <v>6.23719186862E11</v>
+      </c>
+      <c r="R29" s="13" t="s">
+        <v>292</v>
+      </c>
+      <c r="S29" s="12" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30" ht="22.5" customHeight="1">
+      <c r="A30" s="11">
+        <v>46259.95316060186</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>293</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>294</v>
+      </c>
+      <c r="D30" s="12">
+        <v>6.290406354E9</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>295</v>
+      </c>
+      <c r="F30" s="12" t="s">
+        <v>296</v>
+      </c>
+      <c r="G30" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="H30" s="12" t="s">
+        <v>297</v>
+      </c>
+      <c r="I30" s="12">
+        <v>3.0</v>
+      </c>
+      <c r="J30" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="K30" s="12" t="s">
+        <v>298</v>
+      </c>
+      <c r="M30" s="12" t="s">
+        <v>299</v>
+      </c>
+      <c r="N30" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="O30" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="P30" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="Q30" s="12" t="s">
+        <v>300</v>
+      </c>
+      <c r="R30" s="13" t="s">
+        <v>301</v>
+      </c>
+      <c r="S30" s="12" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="31" ht="22.5" customHeight="1">
+      <c r="A31" s="2">
         <v>46258.40555555555</v>
       </c>
-      <c r="B24" s="3" t="s">
-        <v>246</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>247</v>
-      </c>
-      <c r="D24" s="3">
+      <c r="B31" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="D31" s="3">
         <v>9.123704457E9</v>
       </c>
-      <c r="E24" s="3" t="s">
-        <v>248</v>
-      </c>
-      <c r="F24" s="3" t="s">
+      <c r="E31" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="F31" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="G24" s="3" t="s">
-        <v>249</v>
-      </c>
-      <c r="H24" s="3" t="s">
-        <v>250</v>
-      </c>
-      <c r="I24" s="3">
+      <c r="G31" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="H31" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="I31" s="3">
         <v>2.0</v>
       </c>
-      <c r="J24" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="K24" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="L24" s="4" t="s">
-        <v>253</v>
-      </c>
-      <c r="M24" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="N24" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="O24" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="P24" s="3" t="s">
-        <v>254</v>
-      </c>
-      <c r="Q24" s="3" t="s">
-        <v>255</v>
-      </c>
-      <c r="R24" s="3"/>
-      <c r="S24" s="3"/>
+      <c r="J31" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="K31" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="L31" s="4" t="s">
+        <v>309</v>
+      </c>
+      <c r="M31" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="N31" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="O31" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="P31" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="Q31" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="R31" s="3"/>
+      <c r="S31" s="3"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2669,11 +3263,18 @@
     <hyperlink r:id="rId27" ref="R22"/>
     <hyperlink r:id="rId28" ref="L23"/>
     <hyperlink r:id="rId29" ref="R23"/>
-    <hyperlink r:id="rId30" ref="L24"/>
+    <hyperlink r:id="rId30" ref="R24"/>
+    <hyperlink r:id="rId31" ref="R25"/>
+    <hyperlink r:id="rId32" ref="R26"/>
+    <hyperlink r:id="rId33" ref="R27"/>
+    <hyperlink r:id="rId34" ref="R28"/>
+    <hyperlink r:id="rId35" ref="R29"/>
+    <hyperlink r:id="rId36" ref="R30"/>
+    <hyperlink r:id="rId37" ref="L31"/>
   </hyperlinks>
-  <drawing r:id="rId31"/>
+  <drawing r:id="rId38"/>
   <tableParts count="1">
-    <tablePart r:id="rId33"/>
+    <tablePart r:id="rId40"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>